<commit_message>
Raise Hyundai SND96 city-color rate to SAR 160/day
160/day beats a flat 20% uplift on the original 168,750 (202,500), so the
per-unit rate wins: 90 units x 15 days x 160 = 216,000 excl. VAT, 248,400
incl. VAT. Removed the goodwill discount line tied to the old 168K target.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TF4abcCWc11H47Q8mehd7k
</commit_message>
<xml_diff>
--- a/Hyundai_SND96_CityColor_Quotation.xlsx
+++ b/Hyundai_SND96_CityColor_Quotation.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Quotation" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Quotation!$A$1:$F$70</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Quotation!$A$1:$F$68</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="76">
   <si>
     <t xml:space="preserve">QUOTATION</t>
   </si>
@@ -148,7 +148,7 @@
     <t xml:space="preserve">Nos</t>
   </si>
   <si>
-    <t xml:space="preserve">Rental for 15 days @ SAR 125 per unit per day</t>
+    <t xml:space="preserve">Rental for 15 days @ SAR 160 per unit per day</t>
   </si>
   <si>
     <t xml:space="preserve">Transportation to Site</t>
@@ -220,13 +220,7 @@
     <t xml:space="preserve">Cost per Showroom</t>
   </si>
   <si>
-    <t xml:space="preserve">Subtotal — All 9 Showrooms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saudi National Day 96 Goodwill Discount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NET TOTAL (excl. VAT)</t>
+    <t xml:space="preserve">TOTAL PROJECT VALUE — All 9 Showrooms (excl. VAT)</t>
   </si>
   <si>
     <t xml:space="preserve">VAT (15%)</t>
@@ -244,7 +238,7 @@
     <t xml:space="preserve">5.  IMPORTANT NOTES &amp; TERMS</t>
   </si>
   <si>
-    <t xml:space="preserve">•  The rate of SAR 125 per City-Color per day is all-inclusive, covering rental, transportation, installation, accessories, testing, commissioning, technical support, dismantling and removal.</t>
+    <t xml:space="preserve">•  The rate of SAR 160 per City-Color per day is all-inclusive, covering rental, transportation, installation, accessories, testing, commissioning, technical support, dismantling and removal.</t>
   </si>
   <si>
     <t xml:space="preserve">•  Pricing is based on standard installation conditions. Any special access requirements (crane, boom lift, scaffolding, special permits, major electrical works, etc.) will be quoted separately after site assessment.</t>
@@ -267,15 +261,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="General"/>
     <numFmt numFmtId="167" formatCode="0"/>
-    <numFmt numFmtId="168" formatCode="#,##0;\(#,##0\)"/>
-    <numFmt numFmtId="169" formatCode="#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -415,14 +408,6 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
@@ -453,7 +438,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -490,12 +475,6 @@
         <bgColor rgb="FFF4FAFA"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF3CD"/>
-        <bgColor rgb="FFF4FAFA"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
@@ -546,7 +525,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -687,31 +666,27 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -744,7 +719,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF3CD"/>
+      <rgbColor rgb="FFF4FAFA"/>
       <rgbColor rgb="FFE8F2F3"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -759,7 +734,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFF4FAFA"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -1009,7 +984,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A2:F70"/>
+  <dimension ref="A2:F68"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1170,11 +1145,11 @@
         <v>15</v>
       </c>
       <c r="E19" s="14" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F19" s="15" t="n">
         <f aca="false">C19*D19*E19</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1191,11 +1166,11 @@
         <v>15</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F20" s="20" t="n">
         <f aca="false">C20*D20*E20</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1212,11 +1187,11 @@
         <v>15</v>
       </c>
       <c r="E21" s="14" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F21" s="15" t="n">
         <f aca="false">C21*D21*E21</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1233,11 +1208,11 @@
         <v>15</v>
       </c>
       <c r="E22" s="19" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F22" s="20" t="n">
         <f aca="false">C22*D22*E22</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1254,11 +1229,11 @@
         <v>15</v>
       </c>
       <c r="E23" s="14" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F23" s="15" t="n">
         <f aca="false">C23*D23*E23</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1275,11 +1250,11 @@
         <v>15</v>
       </c>
       <c r="E24" s="19" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F24" s="20" t="n">
         <f aca="false">C24*D24*E24</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1296,11 +1271,11 @@
         <v>15</v>
       </c>
       <c r="E25" s="14" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F25" s="15" t="n">
         <f aca="false">C25*D25*E25</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1317,11 +1292,11 @@
         <v>15</v>
       </c>
       <c r="E26" s="19" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F26" s="20" t="n">
         <f aca="false">C26*D26*E26</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1338,11 +1313,11 @@
         <v>15</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F27" s="15" t="n">
         <f aca="false">C27*D27*E27</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1362,7 +1337,7 @@
       </c>
       <c r="F28" s="23" t="n">
         <f aca="false">SUM(F19:F27)</f>
-        <v>168750</v>
+        <v>216000</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1678,7 +1653,7 @@
       <c r="D50" s="7"/>
       <c r="E50" s="32" t="n">
         <f aca="false">E19</f>
-        <v>125</v>
+        <v>160</v>
       </c>
       <c r="F50" s="32"/>
     </row>
@@ -1691,7 +1666,7 @@
       <c r="D51" s="7"/>
       <c r="E51" s="32" t="n">
         <f aca="false">E19*15</f>
-        <v>1875</v>
+        <v>2400</v>
       </c>
       <c r="F51" s="32"/>
     </row>
@@ -1704,7 +1679,7 @@
       <c r="D52" s="7"/>
       <c r="E52" s="32" t="n">
         <f aca="false">F19</f>
-        <v>18750</v>
+        <v>24000</v>
       </c>
       <c r="F52" s="32"/>
     </row>
@@ -1717,7 +1692,7 @@
       <c r="D53" s="33"/>
       <c r="E53" s="34" t="n">
         <f aca="false">F28</f>
-        <v>168750</v>
+        <v>216000</v>
       </c>
       <c r="F53" s="34"/>
     </row>
@@ -1729,122 +1704,107 @@
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="35" t="n">
-        <v>-750</v>
+        <f aca="false">ROUND(E53*0.15,2)</f>
+        <v>32400</v>
       </c>
       <c r="F54" s="35"/>
     </row>
-    <row r="55" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="33" t="s">
+    <row r="55" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="B55" s="33"/>
-      <c r="C55" s="33"/>
-      <c r="D55" s="33"/>
-      <c r="E55" s="34" t="n">
-        <f aca="false">F28+E54</f>
-        <v>168000</v>
-      </c>
-      <c r="F55" s="34"/>
-    </row>
-    <row r="56" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="s">
+      <c r="B55" s="36"/>
+      <c r="C55" s="36"/>
+      <c r="D55" s="36"/>
+      <c r="E55" s="37" t="n">
+        <f aca="false">E53+E54</f>
+        <v>248400</v>
+      </c>
+      <c r="F55" s="37"/>
+    </row>
+    <row r="57" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B56" s="7"/>
-      <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="36" t="n">
-        <f aca="false">ROUND(E55*0.15,2)</f>
-        <v>25200</v>
-      </c>
-      <c r="F56" s="36"/>
-    </row>
-    <row r="57" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="37" t="s">
+      <c r="B57" s="9"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+      <c r="F57" s="9"/>
+    </row>
+    <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="B57" s="37"/>
-      <c r="C57" s="37"/>
-      <c r="D57" s="37"/>
-      <c r="E57" s="38" t="n">
-        <f aca="false">E55+E56</f>
-        <v>193200</v>
-      </c>
-      <c r="F57" s="38"/>
-    </row>
-    <row r="59" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="9" t="s">
+      <c r="B58" s="38"/>
+      <c r="C58" s="38"/>
+      <c r="D58" s="38"/>
+      <c r="E58" s="38"/>
+      <c r="F58" s="38"/>
+    </row>
+    <row r="60" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
-    </row>
-    <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="39" t="s">
+      <c r="B60" s="9"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
+    </row>
+    <row r="61" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="B60" s="39"/>
-      <c r="C60" s="39"/>
-      <c r="D60" s="39"/>
-      <c r="E60" s="39"/>
-      <c r="F60" s="39"/>
-    </row>
-    <row r="62" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="9" t="s">
+      <c r="B61" s="39"/>
+      <c r="C61" s="39"/>
+      <c r="D61" s="39"/>
+      <c r="E61" s="39"/>
+      <c r="F61" s="39"/>
+    </row>
+    <row r="62" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="B62" s="9"/>
-      <c r="C62" s="9"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="9"/>
-      <c r="F62" s="9"/>
+      <c r="B62" s="39"/>
+      <c r="C62" s="39"/>
+      <c r="D62" s="39"/>
+      <c r="E62" s="39"/>
+      <c r="F62" s="39"/>
     </row>
     <row r="63" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="40" t="s">
+      <c r="A63" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="B63" s="40"/>
-      <c r="C63" s="40"/>
-      <c r="D63" s="40"/>
-      <c r="E63" s="40"/>
-      <c r="F63" s="40"/>
-    </row>
-    <row r="64" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="40" t="s">
+      <c r="B63" s="39"/>
+      <c r="C63" s="39"/>
+      <c r="D63" s="39"/>
+      <c r="E63" s="39"/>
+      <c r="F63" s="39"/>
+    </row>
+    <row r="64" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="B64" s="40"/>
-      <c r="C64" s="40"/>
-      <c r="D64" s="40"/>
-      <c r="E64" s="40"/>
-      <c r="F64" s="40"/>
-    </row>
-    <row r="65" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="40" t="s">
+      <c r="B64" s="39"/>
+      <c r="C64" s="39"/>
+      <c r="D64" s="39"/>
+      <c r="E64" s="39"/>
+      <c r="F64" s="39"/>
+    </row>
+    <row r="65" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="B65" s="40"/>
-      <c r="C65" s="40"/>
-      <c r="D65" s="40"/>
-      <c r="E65" s="40"/>
-      <c r="F65" s="40"/>
-    </row>
-    <row r="66" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="40" t="s">
+      <c r="B65" s="39"/>
+      <c r="C65" s="39"/>
+      <c r="D65" s="39"/>
+      <c r="E65" s="39"/>
+      <c r="F65" s="39"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="40" t="s">
         <v>75</v>
-      </c>
-      <c r="B66" s="40"/>
-      <c r="C66" s="40"/>
-      <c r="D66" s="40"/>
-      <c r="E66" s="40"/>
-      <c r="F66" s="40"/>
-    </row>
-    <row r="67" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="40" t="s">
-        <v>76</v>
       </c>
       <c r="B67" s="40"/>
       <c r="C67" s="40"/>
@@ -1852,26 +1812,16 @@
       <c r="E67" s="40"/>
       <c r="F67" s="40"/>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="41" t="s">
-        <v>77</v>
-      </c>
-      <c r="B69" s="41"/>
-      <c r="C69" s="41"/>
-      <c r="D69" s="41"/>
-      <c r="E69" s="41"/>
-      <c r="F69" s="41"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="41"/>
-      <c r="B70" s="41"/>
-      <c r="C70" s="41"/>
-      <c r="D70" s="41"/>
-      <c r="E70" s="41"/>
-      <c r="F70" s="41"/>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="40"/>
+      <c r="B68" s="40"/>
+      <c r="C68" s="40"/>
+      <c r="D68" s="40"/>
+      <c r="E68" s="40"/>
+      <c r="F68" s="40"/>
     </row>
   </sheetData>
-  <mergeCells count="65">
+  <mergeCells count="61">
     <mergeCell ref="D2:F5"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="A10:F10"/>
@@ -1924,19 +1874,15 @@
     <mergeCell ref="E54:F54"/>
     <mergeCell ref="A55:D55"/>
     <mergeCell ref="E55:F55"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A58:F58"/>
     <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A61:F61"/>
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A63:F63"/>
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A65:F65"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A67:F67"/>
-    <mergeCell ref="A69:F70"/>
+    <mergeCell ref="A67:F68"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.511811023622047" footer="0.5"/>

</xml_diff>

<commit_message>
Add signature and company stamp block to Hyundai SND96 quotation
Generates reusable Miradore stamp and signature PNG assets and places
them in a signing block: authorized signatory with stamp on the left,
client acceptance box for Hyundai on the right.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TF4abcCWc11H47Q8mehd7k
</commit_message>
<xml_diff>
--- a/Hyundai_SND96_CityColor_Quotation.xlsx
+++ b/Hyundai_SND96_CityColor_Quotation.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Quotation" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Quotation!$A$1:$F$68</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Quotation!$A$1:$F$77</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="80">
   <si>
     <t xml:space="preserve">QUOTATION</t>
   </si>
@@ -251,6 +251,18 @@
   </si>
   <si>
     <t xml:space="preserve">•  All prices are in Saudi Riyals (SAR) and exclude 15% VAT, shown separately above.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For &amp; on behalf of — MIRADORE EXPERIENCES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLIENT ACCEPTANCE — HYUNDAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authorized Signatory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signature, Company Stamp &amp; Date</t>
   </si>
   <si>
     <t xml:space="preserve">MIRADORE EXPERIENCES — RIYADH, KINGDOM OF SAUDI ARABIA
@@ -476,7 +488,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -499,6 +511,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF5B6B6E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -525,7 +546,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -684,6 +705,14 @@
     </xf>
     <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -790,6 +819,80 @@
         <a:xfrm>
           <a:off x="444600" y="190440"/>
           <a:ext cx="2857320" cy="780840"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>76320</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>171360</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2124000</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>56880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="520920" y="15211440"/>
+          <a:ext cx="2047680" cy="723600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1428840</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>19080</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2419200</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>171360</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1873440" y="15059160"/>
+          <a:ext cx="990360" cy="990360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -984,7 +1087,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A2:F68"/>
+  <dimension ref="A2:F77"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1802,26 +1905,55 @@
       <c r="E65" s="39"/>
       <c r="F65" s="39"/>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="40" t="s">
         <v>75</v>
       </c>
       <c r="B67" s="40"/>
       <c r="C67" s="40"/>
-      <c r="D67" s="40"/>
+      <c r="D67" s="40" t="s">
+        <v>76</v>
+      </c>
       <c r="E67" s="40"/>
       <c r="F67" s="40"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="40"/>
-      <c r="B68" s="40"/>
-      <c r="C68" s="40"/>
-      <c r="D68" s="40"/>
-      <c r="E68" s="40"/>
-      <c r="F68" s="40"/>
+    <row r="68" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="69" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="70" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="71" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="72" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="B74" s="41"/>
+      <c r="D74" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="E74" s="41"/>
+      <c r="F74" s="41"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="B76" s="42"/>
+      <c r="C76" s="42"/>
+      <c r="D76" s="42"/>
+      <c r="E76" s="42"/>
+      <c r="F76" s="42"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="42"/>
+      <c r="B77" s="42"/>
+      <c r="C77" s="42"/>
+      <c r="D77" s="42"/>
+      <c r="E77" s="42"/>
+      <c r="F77" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="61">
+  <mergeCells count="65">
     <mergeCell ref="D2:F5"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="A10:F10"/>
@@ -1882,7 +2014,11 @@
     <mergeCell ref="A63:F63"/>
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A65:F65"/>
-    <mergeCell ref="A67:F68"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="D67:F67"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="D74:F74"/>
+    <mergeCell ref="A76:F77"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.55" header="0.511811023622047" footer="0.5"/>

</xml_diff>

<commit_message>
Use genuine director signature extracted from signed invoice PDF
The signature (with its underline swoosh) is rasterized at 300dpi from the
Riyadh Digital City advance invoice already in the repo and made
transparent. Signatory name corrected to Adeel Ahmed per company documents.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TF4abcCWc11H47Q8mehd7k
</commit_message>
<xml_diff>
--- a/Hyundai_SND96_CityColor_Quotation.xlsx
+++ b/Hyundai_SND96_CityColor_Quotation.xlsx
@@ -247,7 +247,7 @@
     <t xml:space="preserve">CLIENT ACCEPTANCE — HYUNDAI</t>
   </si>
   <si>
-    <t xml:space="preserve">Adeel Ahmad — Director</t>
+    <t xml:space="preserve">Adeel Ahmed — Director</t>
   </si>
   <si>
     <t xml:space="preserve">Signature, Company Stamp &amp; Date</t>
@@ -914,14 +914,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>76320</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>171360</xdr:rowOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>37800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>2124000</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>56520</xdr:rowOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>190080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -934,8 +934,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="520920" y="15496920"/>
-          <a:ext cx="2047680" cy="723600"/>
+          <a:off x="520920" y="15573240"/>
+          <a:ext cx="2047680" cy="571320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Widen columns so the quote fills the full A4 page width
Fit-to-page scaling was height-bound, leaving a white strip on the right;
column widths now match the A4 aspect.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TF4abcCWc11H47Q8mehd7k
</commit_message>
<xml_diff>
--- a/Hyundai_SND96_CityColor_Quotation.xlsx
+++ b/Hyundai_SND96_CityColor_Quotation.xlsx
@@ -897,7 +897,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="444600" y="190440"/>
+          <a:off x="533520" y="190440"/>
           <a:ext cx="2857320" cy="780840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -934,7 +934,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="520920" y="15573240"/>
+          <a:off x="609840" y="15573240"/>
           <a:ext cx="2047680" cy="571320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -971,7 +971,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1778040" y="15344640"/>
+          <a:off x="1866960" y="15344640"/>
           <a:ext cx="1266480" cy="980640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1170,12 +1170,11 @@
   <dimension ref="A2:F78"/>
   <sheetFormatPr defaultColWidth="13" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="7" style="0" width="13"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Reduce city-color rate to SAR 156/day
New totals: 210,600 excl. VAT; 242,190 incl. VAT.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TF4abcCWc11H47Q8mehd7k
</commit_message>
<xml_diff>
--- a/Hyundai_SND96_CityColor_Quotation.xlsx
+++ b/Hyundai_SND96_CityColor_Quotation.xlsx
@@ -139,7 +139,7 @@
     <t xml:space="preserve">Nos</t>
   </si>
   <si>
-    <t xml:space="preserve">Rental for 15 days @ SAR 160 per unit per day</t>
+    <t xml:space="preserve">Rental for 15 days @ SAR 156 per unit per day</t>
   </si>
   <si>
     <t xml:space="preserve">Transportation to Site</t>
@@ -226,7 +226,7 @@
     <t xml:space="preserve">5.  IMPORTANT NOTES &amp; TERMS</t>
   </si>
   <si>
-    <t xml:space="preserve">•  The rate of SAR 160 per City-Color per day is all-inclusive, covering rental, transportation, installation, accessories, testing, commissioning, technical support, dismantling and removal.</t>
+    <t xml:space="preserve">•  The rate of SAR 156 per City-Color per day is all-inclusive, covering rental, transportation, installation, accessories, testing, commissioning, technical support, dismantling and removal.</t>
   </si>
   <si>
     <t xml:space="preserve">•  Pricing is based on standard installation conditions. Any special access requirements (crane, boom lift, scaffolding, special permits, major electrical works, etc.) will be quoted separately after site assessment.</t>
@@ -1322,11 +1322,11 @@
         <v>15</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F19" s="16" t="n">
         <f aca="false">C19*D19*E19</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1343,11 +1343,11 @@
         <v>15</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F20" s="21" t="n">
         <f aca="false">C20*D20*E20</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1364,11 +1364,11 @@
         <v>15</v>
       </c>
       <c r="E21" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F21" s="16" t="n">
         <f aca="false">C21*D21*E21</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1385,11 +1385,11 @@
         <v>15</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F22" s="21" t="n">
         <f aca="false">C22*D22*E22</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1406,11 +1406,11 @@
         <v>15</v>
       </c>
       <c r="E23" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F23" s="16" t="n">
         <f aca="false">C23*D23*E23</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1427,11 +1427,11 @@
         <v>15</v>
       </c>
       <c r="E24" s="20" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F24" s="21" t="n">
         <f aca="false">C24*D24*E24</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1448,11 +1448,11 @@
         <v>15</v>
       </c>
       <c r="E25" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F25" s="16" t="n">
         <f aca="false">C25*D25*E25</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1469,11 +1469,11 @@
         <v>15</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F26" s="21" t="n">
         <f aca="false">C26*D26*E26</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1490,11 +1490,11 @@
         <v>15</v>
       </c>
       <c r="E27" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F27" s="16" t="n">
         <f aca="false">C27*D27*E27</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="F28" s="24" t="n">
         <f aca="false">SUM(F19:F27)</f>
-        <v>216000</v>
+        <v>210600</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1830,7 +1830,7 @@
       <c r="D50" s="31"/>
       <c r="E50" s="34" t="n">
         <f aca="false">E19</f>
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F50" s="34"/>
     </row>
@@ -1843,7 +1843,7 @@
       <c r="D51" s="31"/>
       <c r="E51" s="34" t="n">
         <f aca="false">E19*15</f>
-        <v>2400</v>
+        <v>2340</v>
       </c>
       <c r="F51" s="34"/>
     </row>
@@ -1856,7 +1856,7 @@
       <c r="D52" s="31"/>
       <c r="E52" s="34" t="n">
         <f aca="false">F19</f>
-        <v>24000</v>
+        <v>23400</v>
       </c>
       <c r="F52" s="34"/>
     </row>
@@ -1869,7 +1869,7 @@
       <c r="D53" s="35"/>
       <c r="E53" s="36" t="n">
         <f aca="false">F28</f>
-        <v>216000</v>
+        <v>210600</v>
       </c>
       <c r="F53" s="36"/>
     </row>
@@ -1882,7 +1882,7 @@
       <c r="D54" s="31"/>
       <c r="E54" s="37" t="n">
         <f aca="false">ROUND(E53*0.15,2)</f>
-        <v>32400</v>
+        <v>31590</v>
       </c>
       <c r="F54" s="37"/>
     </row>
@@ -1895,7 +1895,7 @@
       <c r="D55" s="38"/>
       <c r="E55" s="39" t="n">
         <f aca="false">E53+E54</f>
-        <v>248400</v>
+        <v>242190</v>
       </c>
       <c r="F55" s="39"/>
     </row>

</xml_diff>